<commit_message>
Fix scheidungsdrama testakte review findings
</commit_message>
<xml_diff>
--- a/testakten/scheidungsdrama/12_zugewinnausgleich_berechnung.xlsx
+++ b/testakten/scheidungsdrama/12_zugewinnausgleich_berechnung.xlsx
@@ -598,7 +598,7 @@
     <row r="2" ht="30" customHeight="1">
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>Zugewinnausgleich — Wagenknecht / Luetzelberg</t>
+          <t>Zugewinnausgleich — Hanna Trüffelberch / Franz Trüffelberch</t>
         </is>
       </c>
     </row>
@@ -624,12 +624,12 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>Vera Wagenknecht (EUR)</t>
+          <t>Hanna Trüffelberch (EUR)</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>Theo Wagenknecht (EUR)</t>
+          <t>Franz Trüffelberch (EUR)</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
@@ -652,7 +652,7 @@
       </c>
       <c r="E7" s="6" t="inlineStr">
         <is>
-          <t>Vera: Eigenangabe plausibel; Theo: ca. Angabe</t>
+          <t>Hanna: Eigenangabe plausibel; Franz: ca. Angabe</t>
         </is>
       </c>
     </row>
@@ -670,7 +670,7 @@
       </c>
       <c r="E8" s="6" t="inlineStr">
         <is>
-          <t>Vera: PKW wertlos; Theo: Werkswagen (kein Eigentum)</t>
+          <t>Hanna: PKW wertlos; Franz: Werkswagen (kein Eigentum)</t>
         </is>
       </c>
     </row>
@@ -706,7 +706,7 @@
       </c>
       <c r="E10" s="6" t="inlineStr">
         <is>
-          <t>Theo: Restdarlehen Meisterschule</t>
+          <t>Franz: Restdarlehen Meisterschule</t>
         </is>
       </c>
     </row>
@@ -743,12 +743,12 @@
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>Vera (EUR)</t>
+          <t>Hanna (EUR)</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
         <is>
-          <t>Theo (EUR)</t>
+          <t>Franz (EUR)</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
@@ -771,7 +771,7 @@
       </c>
       <c r="E15" s="11" t="inlineStr">
         <is>
-          <t>WP Dreschler, Aug. 2025 (Gesamtwert 1.420 TEUR) / Theo: vorläufig, Unterl. fehlen</t>
+          <t>WP Dreschler, Aug. 2025 (Gesamtwert 1.420 TEUR) / Franz: vorläufig, Unterl. fehlen</t>
         </is>
       </c>
     </row>
@@ -825,7 +825,7 @@
       </c>
       <c r="E18" s="6" t="inlineStr">
         <is>
-          <t>Kontoauszug Aug. 2025 / Theo: Angabe RAin Ganzhorn, unvollst.</t>
+          <t>Kontoauszug Aug. 2025 / Franz: Angabe RAin Ganzhorn, unvollst.</t>
         </is>
       </c>
     </row>
@@ -843,7 +843,7 @@
       </c>
       <c r="E19" s="11" t="inlineStr">
         <is>
-          <t>Depot Aug. 2025 / Theo: keines bekannt</t>
+          <t>Depot Aug. 2025 / Franz: keines bekannt</t>
         </is>
       </c>
     </row>
@@ -861,7 +861,7 @@
       </c>
       <c r="E20" s="6" t="inlineStr">
         <is>
-          <t>BSV Wüstenrot / Theo: keinen</t>
+          <t>BSV Wüstenrot / Franz: keinen</t>
         </is>
       </c>
     </row>
@@ -879,7 +879,7 @@
       </c>
       <c r="E21" s="11" t="inlineStr">
         <is>
-          <t>Audi A4 Schwacke / Theo: VW Transporter + Seat</t>
+          <t>Audi A4 Schwacke / Franz: VW Transporter + Seat</t>
         </is>
       </c>
     </row>
@@ -897,7 +897,7 @@
       </c>
       <c r="E22" s="6" t="inlineStr">
         <is>
-          <t>Kreditkarte / Theo: Privat- + Betriebsschulden (68 TEUR Maschinenkredit ges. = anteilig hier)</t>
+          <t>Kreditkarte / Franz: Privat- + Betriebsschulden (68 TEUR Maschinenkredit ges. = anteilig hier)</t>
         </is>
       </c>
     </row>
@@ -915,7 +915,7 @@
       </c>
       <c r="E23" s="13" t="inlineStr">
         <is>
-          <t>Vera: Summe; Theo: vorläufig (Unterlagen unvollst.)</t>
+          <t>Hanna: Summe; Franz: vorläufig (Unterlagen unvollst.)</t>
         </is>
       </c>
     </row>
@@ -934,12 +934,12 @@
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>Vera (EUR)</t>
+          <t>Hanna (EUR)</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>Theo (EUR)</t>
+          <t>Franz (EUR)</t>
         </is>
       </c>
       <c r="E26" s="4" t="inlineStr">
@@ -976,7 +976,7 @@
       </c>
       <c r="E28" s="6" t="inlineStr">
         <is>
-          <t>Theo AV: neg. → 0</t>
+          <t>Franz AV: neg. → 0</t>
         </is>
       </c>
     </row>
@@ -996,7 +996,7 @@
     <row r="30">
       <c r="B30" s="14" t="inlineStr">
         <is>
-          <t>Differenz Zugewinne (Vera − Theo)</t>
+          <t>Differenz Zugewinne (Hanna − Franz)</t>
         </is>
       </c>
       <c r="C30" s="15" t="n">
@@ -1016,7 +1016,7 @@
     <row r="31">
       <c r="B31" s="14" t="inlineStr">
         <is>
-          <t>Ausgleichsanspruch Theo (50 %)</t>
+          <t>Ausgleichsanspruch Franz (50 %)</t>
         </is>
       </c>
       <c r="C31" s="16" t="n">
@@ -1036,7 +1036,7 @@
     <row r="33" ht="36" customHeight="1">
       <c r="B33" s="17" t="inlineStr">
         <is>
-          <t>⚠  Vorläufige Berechnung. Wert Holzwerkstätten e.K. und PartGmbB-Goodwill sind streitig. Bürobewertung kann von 900 TEUR bis 1,5 Mio. EUR variieren. Jahresabschlüsse Theo noch nicht vollständig vorliegend.</t>
+          <t>⚠  Vorläufige Berechnung. Wert Holzwerkstätten e.K. und PartGmbB-Goodwill sind streitig. Bürobewertung kann von 900 TEUR bis 1,5 Mio. EUR variieren. Jahresabschlüsse Franz noch nicht vollständig vorliegend.</t>
         </is>
       </c>
     </row>
@@ -1084,17 +1084,17 @@
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>Veras Anteil 50 % (EUR)</t>
+          <t>Hannas Anteil 50 % (EUR)</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>Veras Zugewinn (EUR)</t>
+          <t>Hannas Zugewinn (EUR)</t>
         </is>
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t>Ausgleich an Theo (EUR)</t>
+          <t>Ausgleich an Franz (EUR)</t>
         </is>
       </c>
     </row>

</xml_diff>